<commit_message>
Quiz answers by closed set; Say hidden until a language reaches 80%; LoRA notebook ready (needs the Kaggle secret)
- POST /asr/choose: the audio is scored against each allowed answer (letter
  names in the UI language and English, yes/no, true/false) with the NCAIR1
  Whisper models; below a 0.6 cut-off (fixed beforehand) "not sure", asked
  again. Synthetic clips: English 42% -> 79%, Hausa 18% -> 51%, Yoruba
  13% -> 58%, Igbo 1% -> 28% right.
- No language reaches 80%, so the quiz hides Say and taps by default
  everywhere; the confirm step stays.
- Magana LoRA notebook: clones outside the output folder; first Kaggle run
  stopped at the HF_TOKEN secret, which must be attached to the notebook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data_sources_tracker.xlsx
+++ b/docs/data_sources_tracker.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Number and unit word lists</t>
+          <t>Number and unit word lists; quiz answer forms</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
-          <t>content/number_words/ (repo)</t>
+          <t>content/number_words/, content/answers/closed_sets.json (repo)</t>
         </is>
       </c>
       <c r="F30" s="19" t="inlineStr">
@@ -3154,20 +3154,23 @@
       <c r="N35" s="13" t="n"/>
     </row>
     <row r="36">
-      <c r="L36" t="inlineStr">
+      <c r="L36" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="M36">
+      <c r="M36" s="13">
         <f>SUM(M2:M34)</f>
         <v/>
       </c>
-      <c r="N36">
+      <c r="N36" s="13">
         <f>SUM(N2:N34)</f>
         <v/>
       </c>
     </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <autoFilter ref="A1:O25"/>
   <dataValidations count="2">
@@ -7230,7 +7233,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36">
+      <c r="A36" s="13">
         <f>IF(LEFT(Sources!H34,3)="Yes",Sources!B34&amp;" — "&amp;Sources!J34&amp;" — "&amp;Sources!E34,"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Accounts: teacher email sign-in, schools and roles, hashed 6-digit codes, class link with portal consent, remove/move/delete learners, audit log; portal Home, Teachers, Learner, Register (state + LGA combobox), team approvals; quizzes owned by teachers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data_sources_tracker.xlsx
+++ b/docs/data_sources_tracker.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -3149,28 +3149,92 @@
       </c>
     </row>
     <row r="35">
-      <c r="L35" s="13" t="n"/>
-      <c r="M35" s="13" t="n"/>
-      <c r="N35" s="13" t="n"/>
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>S34</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Nigeria's states and local government areas (36 states + FCT, 774 LGAs)</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Reference data (places)</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>English (place names)</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/xosasx/nigerian-local-government-areas</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>MIT (© 2022 Osas Obazee); state codes ISO 3166-2:NG; LGA codes Magana's own (NG-LA-IKEJA); Wikidata IDs kept (CC0), 3 of them shared by same-name LGAs in two states</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>Verified 25 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>Yes, with the MIT notice (content/places/LICENSE-ng-lgas.txt)</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>State and LGA pickers (school registration and anywhere Magana asks for a location), stored as codes</t>
+        </is>
+      </c>
+      <c r="J35" s="13" t="inlineStr">
+        <is>
+          <t>Nigerian LGAs by Osas Obazee, MIT licence; Wikidata</t>
+        </is>
+      </c>
+      <c r="K35" s="13" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L35" s="13" t="inlineStr">
+        <is>
+          <t>In use: content/places/ng_states_lgas.json</t>
+        </is>
+      </c>
+      <c r="O35" s="13" t="inlineStr">
+        <is>
+          <t>Counts checked by backend/tests/test_places.py: 37 states and FCT, 774 LGAs, per-state counts (e.g. Lagos 20, Kano 44).</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="L36" s="13" t="inlineStr">
+      <c r="L36" s="13" t="n"/>
+      <c r="M36" s="13" t="n"/>
+      <c r="N36" s="13" t="n"/>
+    </row>
+    <row r="37">
+      <c r="L37" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="M36" s="13">
+      <c r="M37" s="13">
         <f>SUM(M2:M34)</f>
         <v/>
       </c>
-      <c r="N36" s="13">
+      <c r="N37" s="13">
         <f>SUM(N2:N34)</f>
         <v/>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <autoFilter ref="A1:O25"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
White paper reading fixes: two-column pages read column by column with headings and Next column (layout.py); Hausa/Yorùbá/Igbo pages warned once, Yorùbá and Igbo read again with better Tesseract models, words that may have lost a special letter marked and spelled, never changed (letters.py, CC BY-SA word lists); offline basic reading on the phone with ML Kit, number safety kept, encrypted queue for the full reading; capture tilt and blur cues, cut-off text reported; measured before/after (FINDINGS)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data_sources_tracker.xlsx
+++ b/docs/data_sources_tracker.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -3216,21 +3216,382 @@
       </c>
     </row>
     <row r="36">
-      <c r="L36" s="13" t="n"/>
-      <c r="M36" s="13" t="n"/>
-      <c r="N36" s="13" t="n"/>
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>S35</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Wikipedia in Hausa, Yorùbá and Igbo</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Public text (encyclopaedia)</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Hausa, Yorùbá, Igbo</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>https://ha.wikipedia.org · https://yo.wikipedia.org · https://ig.wikipedia.org</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>Verified 26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>Yes, share-alike</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>10 article extracts per language for the letter test (benchmark/letters/, with each article's link); word frequencies from the dumps of 26 Oct 2026 for the word lists (content/word_lists/)</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
+        <is>
+          <t>Text from Hausa, Yorùbá and Igbo Wikipedia, CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L36" s="13" t="inlineStr">
+        <is>
+          <t>In use: 30 extracts; 3 word lists</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="13" t="inlineStr">
+        <is>
+          <t>Test pages are drawn, not photographed: not in the capture log. Word lists are derived works, CC BY-SA 4.0; not reviewed by native speakers.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>S36</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>English Wiktionary: Hausa, Yoruba and Igbo entries (kaikki.org extracts; Category:Igbo lemmas)</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Public dictionary</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>Hausa, Yorùbá, Igbo</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>https://kaikki.org/dictionary/ · https://en.wiktionary.org/wiki/Category:Igbo_lemmas</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0 (and GFDL)</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>Verified 26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>Yes, share-alike</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>Words with special letters for the letter check (content/word_lists/)</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr">
+        <is>
+          <t>Wiktionary contributors, CC BY-SA 4.0; extracts by kaikki.org</t>
+        </is>
+      </c>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
       <c r="L37" s="13" t="inlineStr">
         <is>
+          <t>In use: 3 word lists</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="13" t="inlineStr">
+        <is>
+          <t>Kept only where the spelling is at least 25% of the word's uses in that Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>S37</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Team-written two-column textbook-style pages</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Own content</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>benchmark/columns/pages.json</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>Our own, released CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>N/A, our own</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>Two-column reading order and headings (scripts/column_order_test.py)</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr">
+        <is>
+          <t>Magana Learn team, CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="K38" s="13" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L38" s="13" t="inlineStr">
+        <is>
+          <t>In use: 10 pages</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>10</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="13" t="inlineStr">
+        <is>
+          <t>Drawn, not photographed. Real photographed textbook pages still to come.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>S38</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Tesseract tessdata_fast: yor and script/Latin models</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Model (OCR)</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Yorùbá; Latin-script languages</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/tesseract-ocr/tessdata_fast</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>Verified 26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>Reading Yorùbá and Igbo pages again so fewer special letters are lost (backend/Dockerfile, pinned)</t>
+        </is>
+      </c>
+      <c r="J39" s="13" t="inlineStr">
+        <is>
+          <t>Tesseract OCR tessdata_fast, Apache-2.0</t>
+        </is>
+      </c>
+      <c r="K39" s="13" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L39" s="13" t="inlineStr">
+        <is>
+          <t>In use</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="13" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>S39</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Google ML Kit Text Recognition v2 (Latin, bundled)</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Model (OCR, on the phone)</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Latin-script languages</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>https://developers.google.com/ml-kit/vision/text-recognition/v2</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>Google ML Kit terms (free; proprietary SDK)</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>Verified 26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Ships inside the app; not redistributed separately</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>Offline basic reading on the phone (app/lib/offline/)</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr">
+        <is>
+          <t>Text recognition by Google ML Kit</t>
+        </is>
+      </c>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L40" s="13" t="inlineStr">
+        <is>
+          <t>In use</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="13" t="inlineStr">
+        <is>
+          <t>Bundled model: nothing is downloaded or sent when reading offline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="L41" s="13" t="n"/>
+      <c r="M41" s="13" t="n"/>
+      <c r="N41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="L42" s="13" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="M37" s="13">
+      <c r="M42" s="13">
         <f>SUM(M2:M34)</f>
         <v/>
       </c>
-      <c r="N37" s="13">
+      <c r="N42" s="13">
         <f>SUM(N2:N34)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
0.1.0+8: camera photos 1080 px wide at JPEG q85, shrunk and turned upright on the phone (1600 measured no better); server applies EXIF orientation; no "some lines look handwritten" claim from OCR doubt alone (barcodes skipped, specks and fine print not judged; per-line handwriting rules unchanged); stricter handwriting on health papers (a neatly handwritten dose is never read); grouped warnings (page summary, "unclear" at the spot, "what's unclear?" for the full list; number safety unchanged); newer tips held back for older apps; offline faint-print retry; handwriting test samples (public-domain letter, Caveat OFL) credited (FINDINGS)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data_sources_tracker.xlsx
+++ b/docs/data_sources_tracker.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -3276,10 +3276,10 @@
           <t>In use: 30 extracts; 3 word lists</t>
         </is>
       </c>
-      <c r="M36" t="n">
+      <c r="M36" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N36" t="n">
+      <c r="N36" s="13" t="n">
         <v>0</v>
       </c>
       <c r="O36" s="13" t="inlineStr">
@@ -3349,10 +3349,10 @@
           <t>In use: 3 word lists</t>
         </is>
       </c>
-      <c r="M37" t="n">
+      <c r="M37" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N37" t="n">
+      <c r="N37" s="13" t="n">
         <v>0</v>
       </c>
       <c r="O37" s="13" t="inlineStr">
@@ -3422,10 +3422,10 @@
           <t>In use: 10 pages</t>
         </is>
       </c>
-      <c r="M38" t="n">
+      <c r="M38" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="N38" t="n">
+      <c r="N38" s="13" t="n">
         <v>0</v>
       </c>
       <c r="O38" s="13" t="inlineStr">
@@ -3495,10 +3495,10 @@
           <t>In use</t>
         </is>
       </c>
-      <c r="M39" t="n">
+      <c r="M39" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N39" t="n">
+      <c r="N39" s="13" t="n">
         <v>0</v>
       </c>
       <c r="O39" s="13" t="inlineStr"/>
@@ -3564,10 +3564,10 @@
           <t>In use</t>
         </is>
       </c>
-      <c r="M40" t="n">
+      <c r="M40" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N40" t="n">
+      <c r="N40" s="13" t="n">
         <v>0</v>
       </c>
       <c r="O40" s="13" t="inlineStr">
@@ -3577,21 +3577,167 @@
       </c>
     </row>
     <row r="41">
-      <c r="L41" s="13" t="n"/>
-      <c r="M41" s="13" t="n"/>
-      <c r="N41" s="13" t="n"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>S40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Handwritten letter by Wilbur Underhill Jr. (two sides), Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Public image (handwriting)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>English (1930s cursive)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Handwritten_letter_by_Wilbur_Underhill_Jr._-_Side_A.jpg</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Public domain</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Verified 27 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Handwriting tests (backend/tests/fixtures/handwriting/)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Wilbur Underhill Jr., public domain, via Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>In use: 2 images</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Not part of the benchmark.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="L42" s="13" t="inlineStr">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>S41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Caveat font (Google Fonts)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Font</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Latin script</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://github.com/google/fonts/tree/main/ofl/caveat</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SIL Open Font License 1.1</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Verified 27 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Drawn print-style handwriting for tests (backend/tests/fixtures/fonts/Caveat.ttf)</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Caveat, Copyright 2014 The Caveat Project Authors, SIL OFL 1.1</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>In use: test font</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Drawn handwriting, not a person's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="L43" s="13" t="n"/>
+      <c r="M43" s="13" t="n"/>
+      <c r="N43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="L44" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="M42" s="13">
+      <c r="M44" s="13">
         <f>SUM(M2:M34)</f>
         <v/>
       </c>
-      <c r="N42" s="13">
+      <c r="N44" s="13">
         <f>SUM(N2:N34)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
0.1.0+9: tilt is a tip only and never blocks capture (4 s rule with or without a page, hand-shake grace); server straightens tilted photos (±15°); fix a sharp card read twice by faint recovery; blank photos never turned; diagnostics show why each line is unclear and every utterance's text and timing; script-font church card regression tests (Dancing Script OFL, S42) (FINDINGS)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data_sources_tracker.xlsx
+++ b/docs/data_sources_tracker.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -3577,167 +3577,240 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>S40</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>Handwritten letter by Wilbur Underhill Jr. (two sides), Wikimedia Commons</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>Public image (handwriting)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>English (1930s cursive)</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="13" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Handwritten_letter_by_Wilbur_Underhill_Jr._-_Side_A.jpg</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="13" t="inlineStr">
         <is>
           <t>Public domain</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="13" t="inlineStr">
         <is>
           <t>Verified 27 Oct 2026</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="13" t="inlineStr">
         <is>
           <t>Handwriting tests (backend/tests/fixtures/handwriting/)</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41" s="13" t="inlineStr">
         <is>
           <t>Wilbur Underhill Jr., public domain, via Wikimedia Commons</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="13" t="inlineStr">
         <is>
           <t>Daniel</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L41" s="13" t="inlineStr">
         <is>
           <t>In use: 2 images</t>
         </is>
       </c>
-      <c r="M41" t="n">
+      <c r="M41" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N41" t="n">
+      <c r="N41" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="O41" s="13" t="inlineStr">
         <is>
           <t>Not part of the benchmark.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>S41</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>Caveat font (Google Fonts)</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="13" t="inlineStr">
         <is>
           <t>Font</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="13" t="inlineStr">
         <is>
           <t>Latin script</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="13" t="inlineStr">
         <is>
           <t>https://github.com/google/fonts/tree/main/ofl/caveat</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="13" t="inlineStr">
         <is>
           <t>SIL Open Font License 1.1</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="13" t="inlineStr">
         <is>
           <t>Verified 27 Oct 2026</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I42" s="13" t="inlineStr">
         <is>
           <t>Drawn print-style handwriting for tests (backend/tests/fixtures/fonts/Caveat.ttf)</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J42" s="13" t="inlineStr">
         <is>
           <t>Caveat, Copyright 2014 The Caveat Project Authors, SIL OFL 1.1</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K42" s="13" t="inlineStr">
         <is>
           <t>Daniel</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L42" s="13" t="inlineStr">
         <is>
           <t>In use: test font</t>
         </is>
       </c>
-      <c r="M42" t="n">
+      <c r="M42" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N42" t="n">
+      <c r="N42" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="O42" s="13" t="inlineStr">
         <is>
           <t>Drawn handwriting, not a person's.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="L43" s="13" t="n"/>
-      <c r="M43" s="13" t="n"/>
-      <c r="N43" s="13" t="n"/>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>S42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Dancing Script font (Google Fonts)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Font</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Latin script</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://github.com/google/fonts/tree/main/ofl/dancingscript</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>SIL Open Font License 1.1</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Verified 27 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Drawing a decorative script-print church card for tests (backend/tests/fixtures/fonts/DancingScript.ttf)</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Dancing Script, Copyright 2016 The Dancing Script Project Authors, SIL OFL 1.1</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>In use: test font</t>
+        </is>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Printed script type, not handwriting.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="L44" s="13" t="inlineStr">
+      <c r="L44" s="13" t="n"/>
+      <c r="M44" s="13" t="n"/>
+      <c r="N44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="L45" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="M44" s="13">
+      <c r="M45" s="13">
         <f>SUM(M2:M34)</f>
         <v/>
       </c>
-      <c r="N44" s="13">
+      <c r="N45" s="13">
         <f>SUM(N2:N34)</f>
         <v/>
       </c>

</xml_diff>